<commit_message>
Modified the PropagationControl object to assign a default value for the azimuth of fracture set zero which will be used if the load tensors for all deformation episodes are isotropic, and modified main() (for the standalone version) and ExecuteSimple() (for the Petrel plugin) to set this to the specified minimum horizontal strain azimuth for the first deformation episode. This prevents the fracture orienation defaulting to E-W if another minimum horizontal strain orientation is specified but the strain load is isotropic (B90).
Also added DFM_Plotter_6set_Centrelines.xlsm to data analysis spreadsheet collection.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56D33A9-8DF0-4D1F-BC88-AB5BD6639530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC132EC9-5B33-4634-B6FF-461D46EBCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1167" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="595">
   <si>
     <t>Type</t>
   </si>
@@ -1996,6 +1996,15 @@
   </si>
   <si>
     <t>When run with oblique fracture sets, it occasionally still produces "spiking" factures (where one or more cornerpoints lies way outside the model bounds). This is due to trying to bevel against a nearly parallel intersecting fracture segment edges. Rewritten MacrofractureXYZ.PopulateData() and PointXYZ.getCrossoverPoint() to allow limits to the bevelling relative to the fracture segment against which it is bevelled (both for intersecting fractures and other segments of the same fracture), and incorporate the minimum angle cutoff check into PointXYZ.getCrossoverPoint().</t>
+  </si>
+  <si>
+    <t>B90</t>
+  </si>
+  <si>
+    <t>Setting fracture orientation to E-W if isotropic horizontal strain load is defined</t>
+  </si>
+  <si>
+    <t>If the horizontal strain load is isotropic, the azimuth of set 0 fractures will be set to zero degrees (i.e. E-W striking fractures) even if a different ehmin azimuth is specified. This is because it takes the orientation from minimum principal component of the strain (or stress) load tensor, which gives an azimuth of 0 by default if the tensor is isotropic. This can be solved by assigning a default value in the PropagationControl object which will be used if the load tensors for all deformation episodes are isotropic, and setting this to the specified minimum horizontal strain azimuth for the first deformation episode.</t>
   </si>
 </sst>
 </file>
@@ -2424,7 +2433,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4745,6 +4754,29 @@
         <v>36</v>
       </c>
       <c r="I96" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="F97" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I97" s="3" t="s">
         <v>562</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modified DFMGenerator_Workstep Arguments.ResetDefaults() function to correctly reset values for InitialMicrofractureSizeDistribution_default,InitialStressRelaxation, EhminAzi_default and EhminRate_default, and to set the argument_SimulationCaseN objects to null and clear the argument_SimulationCase_extras array (B91). Also generated Pip installer for Petrel 2024 and updated ReadMe.MD to link to it. Not yet tested.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC132EC9-5B33-4634-B6FF-461D46EBCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{813D3227-383A-4BBA-BC73-712FDB6D5C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="598">
   <si>
     <t>Type</t>
   </si>
@@ -2005,6 +2005,15 @@
   </si>
   <si>
     <t>If the horizontal strain load is isotropic, the azimuth of set 0 fractures will be set to zero degrees (i.e. E-W striking fractures) even if a different ehmin azimuth is specified. This is because it takes the orientation from minimum principal component of the strain (or stress) load tensor, which gives an azimuth of 0 by default if the tensor is isotropic. This can be solved by assigning a default value in the PropagationControl object which will be used if the load tensors for all deformation episodes are isotropic, and setting this to the specified minimum horizontal strain azimuth for the first deformation episode.</t>
+  </si>
+  <si>
+    <t>B91</t>
+  </si>
+  <si>
+    <t>Petrel plugin UI resets input parameters incorrectly</t>
+  </si>
+  <si>
+    <t>If you click the "Reset to defaults" button on the Petrel plugin UI dialog, it resets the Initial microfracture size distribution coefficient value to 2 instead of 3, and the Initial stress relaxation to 1 instead of 0.5. This is because the initialisation values in the DFMGenerator_Workstep Arguments class (lines 5248-5525) were updated to reflect new defaults but the values in the Arguments.ResetDefaults() function were not. Also, Arguments.ResetDefaults() was incorrectly resetting EhminAzi_default and EhminRate_default, and not setting the argument_SimulationCaseN objects to null or clearing the argument_SimulationCase_extras array.</t>
   </si>
 </sst>
 </file>
@@ -2433,7 +2442,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4777,6 +4786,29 @@
         <v>38</v>
       </c>
       <c r="I97" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="F98" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I98" s="3" t="s">
         <v>562</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated to remove redundant arrows on DFMGenerator and DeformationEpisode dialogs (B91). Recomplied and tested Pip installers.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC132EC9-5B33-4634-B6FF-461D46EBCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D413F70-6D8D-4805-8DF3-CDCE52CDD202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="598">
   <si>
     <t>Type</t>
   </si>
@@ -2005,6 +2005,15 @@
   </si>
   <si>
     <t>If the horizontal strain load is isotropic, the azimuth of set 0 fractures will be set to zero degrees (i.e. E-W striking fractures) even if a different ehmin azimuth is specified. This is because it takes the orientation from minimum principal component of the strain (or stress) load tensor, which gives an azimuth of 0 by default if the tensor is isotropic. This can be solved by assigning a default value in the PropagationControl object which will be used if the load tensors for all deformation episodes are isotropic, and setting this to the specified minimum horizontal strain azimuth for the first deformation episode.</t>
+  </si>
+  <si>
+    <t>B91</t>
+  </si>
+  <si>
+    <t>Remove superfluous arrows on Petrel dialogs</t>
+  </si>
+  <si>
+    <t>The Petrel DFM Generator and Deformation episode dialog boxes have arrows in the top right corner which do not do anything. They can be removed by setting the ShowTabListButton properties for the tab controls on these dialogs to false.</t>
   </si>
 </sst>
 </file>
@@ -2433,7 +2442,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4777,6 +4786,29 @@
         <v>38</v>
       </c>
       <c r="I97" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="F98" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I98" s="3" t="s">
         <v>562</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Recompiled standalone version and updated defaults
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7CFDF0-0409-403F-B7E1-6B725E37E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0D6E82-C1C4-442E-BFA9-3959FB173993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -2046,10 +2046,10 @@
     <t>Incorrectly calculating initial horizontal stress if Biot's Coefficient &lt;1</t>
   </si>
   <si>
-    <t>The code was not taking account of differential compaction of grains and matrix when calculating the initial horizontal effective stress when Biot's coefficient &lt; 1. Amongst other issues, this meant that if the initial state was set to critical. It would start in a state of failure.</t>
-  </si>
-  <si>
     <t>Done; needs testing</t>
+  </si>
+  <si>
+    <t>The code was not taking account of differential compaction of grains and matrix when calculating the initial horizontal effective stress when Biot's coefficient &lt; 1. Amongst other issues, this meant that if the initial state was set to critical, it would start in a state of failure.</t>
   </si>
 </sst>
 </file>
@@ -4836,7 +4836,7 @@
         <v>607</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F98" s="6">
         <v>0.5</v>
@@ -4845,7 +4845,7 @@
         <v>36</v>
       </c>
       <c r="I98" s="6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added functionality to calculate and output sigma factors (fracture-bounded block dimensions) (ME64)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0D6E82-C1C4-442E-BFA9-3959FB173993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E070EA-229F-4896-9971-108CDE240D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="613">
   <si>
     <t>Type</t>
   </si>
@@ -2050,6 +2050,15 @@
   </si>
   <si>
     <t>The code was not taking account of differential compaction of grains and matrix when calculating the initial horizontal effective stress when Biot's coefficient &lt; 1. Amongst other issues, this meant that if the initial state was set to critical, it would start in a state of failure.</t>
+  </si>
+  <si>
+    <t>ME64</t>
+  </si>
+  <si>
+    <t>Calculate Sigma factors</t>
+  </si>
+  <si>
+    <t>Calculate sigma factors along with fracture permeability tensors, as defined in Warren &amp; Root 1963 (SPE426) and Kazemi et al. 1976 (SPE5719).</t>
   </si>
 </sst>
 </file>
@@ -4859,7 +4868,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6176,6 +6185,29 @@
         <v>36</v>
       </c>
       <c r="I56" s="6" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="F57" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I57" s="6" t="s">
         <v>605</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modified to calculate the mean connections per macrofracture for each set (ME65). Not yet tested.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E070EA-229F-4896-9971-108CDE240D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCBFA0C-4CCA-4A83-8B52-9ECE952EDA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="616">
   <si>
     <t>Type</t>
   </si>
@@ -2059,6 +2059,15 @@
   </si>
   <si>
     <t>Calculate sigma factors along with fracture permeability tensors, as defined in Warren &amp; Root 1963 (SPE426) and Kazemi et al. 1976 (SPE5719).</t>
+  </si>
+  <si>
+    <t>ME65</t>
+  </si>
+  <si>
+    <t>The code already calculates and outputs mean connections per macrofracture (including fractures from other sets that terminate against the macrocrofracture) for all macrofractures; this is relatively easy since the total number of macrofractures terminating against all other macrofractures is equal to the total number of intersecting tips. However to calculate this per fracture set, we need to know the mean number of fractures from other sets that terminate against fractures of a specific set. This data is stored in the GridblockConfiguration.MFTerminations array</t>
+  </si>
+  <si>
+    <t>Calculate mean connections per macrofracture for each set</t>
   </si>
 </sst>
 </file>
@@ -4868,7 +4877,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6208,6 +6217,29 @@
         <v>36</v>
       </c>
       <c r="I57" s="6" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="F58" s="6">
+        <v>1</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I58" s="6" t="s">
         <v>605</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modified uF and MF size and connectivity corrected permeability functions to include fractures from other dipsets in the same set when calculating distance to the nearest fracture. Also modified fds.calculateCumulativeMicrofracturePopulationArrays() and calculateTotalMicrofracturePopulation() fns to include other fracture dipsets in the same set when calculating distance to the nearest fracture set.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCBFA0C-4CCA-4A83-8B52-9ECE952EDA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05275084-A478-45F9-93CE-F36649030144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="619">
   <si>
     <t>Type</t>
   </si>
@@ -2068,6 +2068,15 @@
   </si>
   <si>
     <t>Calculate mean connections per macrofracture for each set</t>
+  </si>
+  <si>
+    <t>B92</t>
+  </si>
+  <si>
+    <t>Not calculating increment in static microfracture popultion when driving stress is zero</t>
+  </si>
+  <si>
+    <t>When the driving stress is zero, and gamma^(1/beta) is zero, the fds.calculateTotalMicrofracturePopulation() was not incrementing the static microfracture population, even though microfractures could still be deactivated by growth of stress shadows around macrofractures from other dipsets. Active microfracture density was decreased, so total microfracture density was decreasing in inactive fracture dipsets. This was fixed by modifying the fds.calculateTotalMicrofracturePopulation() function to calculate s_uFP30 increment even if ts_gamma_InvBeta_N is zero.</t>
   </si>
 </sst>
 </file>
@@ -2496,7 +2505,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4863,6 +4872,29 @@
         <v>36</v>
       </c>
       <c r="I98" s="6" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A99" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="F99" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I99" s="6" t="s">
         <v>608</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tested Size and Connectivity Corrected permeability tensors to check they are correctly implementing the documented algorithm. Recompiled standalone code and updated the test models to output fracture permeability tensors.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05275084-A478-45F9-93CE-F36649030144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC9B719-4CC4-42CA-884D-C941EAB5D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="622">
   <si>
     <t>Type</t>
   </si>
@@ -1880,9 +1880,6 @@
     <t>Completed in separate document</t>
   </si>
   <si>
-    <t>Requires funding</t>
-  </si>
-  <si>
     <t>Add code to implement algorithm for calculating fracture propagation across layer boundaries in a multilayered section, as described in D9. Initial stage only models propagation upwards from a brittle, stiff reservoir layer into a more compliant topseal with uniform applied strain (AF3a). Later we can implement full multilayer functionality with fractures propagating upwards and downwards (AF3b) and fracture propagation with arbitrary strain and driving stress in each layer (AF3c).</t>
   </si>
   <si>
@@ -2046,9 +2043,6 @@
     <t>Incorrectly calculating initial horizontal stress if Biot's Coefficient &lt;1</t>
   </si>
   <si>
-    <t>Done; needs testing</t>
-  </si>
-  <si>
     <t>The code was not taking account of differential compaction of grains and matrix when calculating the initial horizontal effective stress when Biot's coefficient &lt; 1. Amongst other issues, this meant that if the initial state was set to critical, it would start in a state of failure.</t>
   </si>
   <si>
@@ -2077,6 +2071,21 @@
   </si>
   <si>
     <t>When the driving stress is zero, and gamma^(1/beta) is zero, the fds.calculateTotalMicrofracturePopulation() was not incrementing the static microfracture population, even though microfractures could still be deactivated by growth of stress shadows around macrofractures from other dipsets. Active microfracture density was decreased, so total microfracture density was decreasing in inactive fracture dipsets. This was fixed by modifying the fds.calculateTotalMicrofracturePopulation() function to calculate s_uFP30 increment even if ts_gamma_InvBeta_N is zero.</t>
+  </si>
+  <si>
+    <t>Update doucmentation for v2.3</t>
+  </si>
+  <si>
+    <t>Update run-through guide for v2.3 - especially section on outputting permeability tensors</t>
+  </si>
+  <si>
+    <t>D22</t>
+  </si>
+  <si>
+    <t>Done in geothermal version (2.4) as part of Go-Forward project (ME62-65)</t>
+  </si>
+  <si>
+    <t>Work underway as part of Go-Forward project</t>
   </si>
 </sst>
 </file>
@@ -2119,7 +2128,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2152,12 +2161,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -2175,7 +2178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2214,12 +2217,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2715,7 +2712,7 @@
         <v>36</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3039,7 +3036,7 @@
         <v>38</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3493,7 +3490,7 @@
         <v>261</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F43" s="3">
         <v>0.25</v>
@@ -4104,13 +4101,13 @@
         <v>443</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F68" s="3">
         <v>1</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H68" s="3" t="s">
         <v>36</v>
@@ -4136,7 +4133,7 @@
         <v>0.25</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>36</v>
@@ -4162,7 +4159,7 @@
         <v>0.25</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>36</v>
@@ -4188,7 +4185,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H71" s="3" t="s">
         <v>36</v>
@@ -4214,7 +4211,7 @@
         <v>0.25</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>36</v>
@@ -4240,7 +4237,7 @@
         <v>0.25</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>36</v>
@@ -4266,7 +4263,7 @@
         <v>0.25</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>36</v>
@@ -4428,7 +4425,7 @@
         <v>36</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="81" spans="1:9" s="3" customFormat="1" ht="120" x14ac:dyDescent="0.25">
@@ -4442,7 +4439,7 @@
         <v>506</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F81" s="3">
         <v>1</v>
@@ -4454,7 +4451,7 @@
         <v>36</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="82" spans="1:9" s="3" customFormat="1" ht="195" x14ac:dyDescent="0.25">
@@ -4468,7 +4465,7 @@
         <v>508</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F82" s="3">
         <v>1</v>
@@ -4480,7 +4477,7 @@
         <v>36</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="83" spans="1:9" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -4506,7 +4503,7 @@
         <v>36</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="84" spans="1:9" s="3" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -4532,7 +4529,7 @@
         <v>36</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="85" spans="1:9" ht="150" x14ac:dyDescent="0.25">
@@ -4558,7 +4555,7 @@
         <v>36</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="86" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -4584,7 +4581,7 @@
         <v>36</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="87" spans="1:9" s="3" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -4610,7 +4607,7 @@
         <v>36</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="88" spans="1:9" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -4636,7 +4633,7 @@
         <v>36</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="89" spans="1:9" s="3" customFormat="1" ht="150" x14ac:dyDescent="0.25">
@@ -4662,7 +4659,7 @@
         <v>36</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="90" spans="1:9" s="3" customFormat="1" ht="135" x14ac:dyDescent="0.25">
@@ -4688,21 +4685,21 @@
         <v>36</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="91" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F91" s="3">
         <v>0.5</v>
@@ -4711,21 +4708,21 @@
         <v>36</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="92" spans="1:9" s="3" customFormat="1" ht="165" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C92" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="B92" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C92" s="4" t="s">
+      <c r="D92" s="4" t="s">
         <v>575</v>
-      </c>
-      <c r="D92" s="4" t="s">
-        <v>576</v>
       </c>
       <c r="F92" s="3">
         <v>1</v>
@@ -4734,21 +4731,21 @@
         <v>36</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="93" spans="1:9" s="3" customFormat="1" ht="150" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C93" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C93" s="4" t="s">
+      <c r="D93" s="4" t="s">
         <v>580</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>581</v>
       </c>
       <c r="F93" s="3">
         <v>0.5</v>
@@ -4757,21 +4754,21 @@
         <v>36</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="94" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C94" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="B94" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C94" s="4" t="s">
+      <c r="D94" s="4" t="s">
         <v>583</v>
-      </c>
-      <c r="D94" s="4" t="s">
-        <v>584</v>
       </c>
       <c r="F94" s="3">
         <v>0.1</v>
@@ -4780,21 +4777,21 @@
         <v>36</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="95" spans="1:9" s="3" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C95" s="4" t="s">
         <v>585</v>
       </c>
-      <c r="B95" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="D95" s="4" t="s">
         <v>586</v>
-      </c>
-      <c r="D95" s="4" t="s">
-        <v>587</v>
       </c>
       <c r="F95" s="3">
         <v>0.5</v>
@@ -4803,21 +4800,21 @@
         <v>36</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="96" spans="1:9" s="3" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F96" s="3">
         <v>0.2</v>
@@ -4826,21 +4823,21 @@
         <v>36</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="97" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C97" s="4" t="s">
         <v>591</v>
       </c>
-      <c r="B97" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C97" s="4" t="s">
+      <c r="D97" s="4" t="s">
         <v>592</v>
-      </c>
-      <c r="D97" s="4" t="s">
-        <v>593</v>
       </c>
       <c r="F97" s="3">
         <v>0.2</v>
@@ -4849,53 +4846,53 @@
         <v>38</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A98" s="6" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
+        <v>605</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>606</v>
       </c>
-      <c r="B98" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C98" s="7" t="s">
+      <c r="D98" s="4" t="s">
         <v>607</v>
       </c>
-      <c r="D98" s="7" t="s">
-        <v>609</v>
-      </c>
-      <c r="F98" s="6">
+      <c r="F98" s="3">
         <v>0.5</v>
       </c>
-      <c r="H98" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I98" s="6" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A99" s="6" t="s">
+      <c r="H98" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" s="3" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A99" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D99" s="4" t="s">
         <v>616</v>
       </c>
-      <c r="B99" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C99" s="7" t="s">
-        <v>617</v>
-      </c>
-      <c r="D99" s="7" t="s">
-        <v>618</v>
-      </c>
-      <c r="F99" s="6">
+      <c r="F99" s="3">
         <v>0.5</v>
       </c>
-      <c r="H99" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I99" s="6" t="s">
-        <v>608</v>
+      <c r="H99" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -5162,7 +5159,7 @@
         <v>421</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -5847,7 +5844,7 @@
         <v>378</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="F39" s="1">
         <v>1</v>
@@ -5890,7 +5887,7 @@
         <v>500</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -5898,7 +5895,7 @@
         <v>501</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="3" customFormat="1" ht="120" x14ac:dyDescent="0.25">
@@ -5953,26 +5950,26 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:9" s="12" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+    <row r="45" spans="1:9" s="3" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="C45" s="4" t="s">
         <v>436</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="F45" s="12">
+      <c r="F45" s="3">
         <v>0.2</v>
       </c>
-      <c r="H45" s="12" t="s">
+      <c r="H45" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I45" s="12" t="s">
+      <c r="I45" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -6065,29 +6062,29 @@
         <v>36</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" s="14" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" s="12" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
         <v>520</v>
       </c>
-      <c r="B50" s="14" t="s">
+      <c r="B50" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="C50" s="13" t="s">
         <v>521</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="D50" s="13" t="s">
         <v>522</v>
       </c>
-      <c r="F50" s="14">
-        <v>3</v>
-      </c>
-      <c r="G50" s="14" t="s">
+      <c r="F50" s="12">
+        <v>3</v>
+      </c>
+      <c r="G50" s="12" t="s">
         <v>523</v>
       </c>
-      <c r="H50" s="14" t="s">
+      <c r="H50" s="12" t="s">
         <v>36</v>
       </c>
     </row>
@@ -6134,7 +6131,7 @@
         <v>38</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="53" spans="1:9" s="3" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -6148,7 +6145,7 @@
         <v>550</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F53" s="3">
         <v>0.5</v>
@@ -6162,16 +6159,16 @@
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C54" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="D54" s="7" t="s">
         <v>597</v>
-      </c>
-      <c r="D54" s="7" t="s">
-        <v>598</v>
       </c>
       <c r="F54" s="6">
         <v>0.5</v>
@@ -6180,21 +6177,21 @@
         <v>38</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C55" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>600</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>601</v>
       </c>
       <c r="F55" s="6">
         <v>2</v>
@@ -6203,21 +6200,21 @@
         <v>36</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C56" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="D56" s="7" t="s">
         <v>603</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>604</v>
       </c>
       <c r="F56" s="6">
         <v>2</v>
@@ -6226,21 +6223,21 @@
         <v>36</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="F57" s="6">
         <v>0.5</v>
@@ -6249,21 +6246,21 @@
         <v>36</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="F58" s="6">
         <v>1</v>
@@ -6272,7 +6269,7 @@
         <v>36</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -6285,7 +6282,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6743,7 +6740,7 @@
         <v>325</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F18" s="3">
         <v>1</v>
@@ -6832,7 +6829,7 @@
         <v>475</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F22" s="3">
         <v>1</v>
@@ -6842,6 +6839,26 @@
       </c>
       <c r="I22" s="3" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>619</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>618</v>
+      </c>
+      <c r="F23" s="8">
+        <v>1</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -6945,29 +6962,29 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="14" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:9" s="12" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="F4" s="12">
+        <v>50</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>554</v>
       </c>
-      <c r="F4" s="14">
-        <v>50</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>555</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="14" t="s">
+      <c r="H4" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="12" t="s">
         <v>415</v>
       </c>
     </row>
@@ -6982,7 +6999,7 @@
         <v>240</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F5" s="3">
         <v>2</v>
@@ -7005,7 +7022,7 @@
         <v>260</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F6" s="3">
         <v>2</v>
@@ -7034,7 +7051,7 @@
         <v>5</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>36</v>
@@ -7083,7 +7100,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>36</v>
@@ -7092,51 +7109,51 @@
         <v>499</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>476</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="6">
         <v>10</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="1" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="I10" s="6" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>515</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="13" t="s">
         <v>516</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="13" t="s">
         <v>517</v>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="12">
         <f>20*12</f>
         <v>240</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="I11" s="14" t="s">
-        <v>553</v>
+      <c r="I11" s="12" t="s">
+        <v>621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new functions to the FCD_list object to calculate an average stress shadow width during the growth of the fracture set, weighted according to MFP32 increase in each timestep, to determine relay zone offsets when calculating MF Size and Connectivity Corrected Permeability (B93). Modified FractureCalculationData.SetEvolutionStage to cache and reset Cum_Gamma_Mminus1 and Cum_HalfLength_Mminus1 when setting gamma_InvBeta_M and Mean_MF_PropagationRate_M to zero (B94)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC9B719-4CC4-42CA-884D-C941EAB5D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCBBA87-2E96-4A29-831E-B033149F7E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="629">
   <si>
     <t>Type</t>
   </si>
@@ -2086,6 +2086,27 @@
   </si>
   <si>
     <t>Work underway as part of Go-Forward project</t>
+  </si>
+  <si>
+    <t>B93</t>
+  </si>
+  <si>
+    <t>Stress shadow width jumping in final timesteps</t>
+  </si>
+  <si>
+    <t>The stress shadow width of certain key fracture dipsets (e.g. the Inclined Hmin set in Test Model B) jumps suddenly in the final few timesteps as the fracture mode switched to dilatant, even though the fractures have stopped growing. This can cause problems if the stress shadow width is used to calculate mean offset of fracture segments (e.g. in the MF Size and Connectivity Corrected Permeability algorithm), as the current stress shadow width used in the calculation will not be the same as that active during fracture growth and controlling the geometry. To get around this, new functions have been added to the FCD_list object to calculate an average stress shadow width during the growth of the fracture set, weighted according to MFP32 increase in each timestep. These functions (and calling functions in the FractureDipSet object) are used to determine relay zone offsets when calculating MF Size and Connectivity Corrected Permeability.</t>
+  </si>
+  <si>
+    <t>Done; needs testing</t>
+  </si>
+  <si>
+    <t>B94</t>
+  </si>
+  <si>
+    <t>Microfracture density jumping to extreme values in oblique fracture models</t>
+  </si>
+  <si>
+    <t>In models with obliques fractures, the uFP30 and uFP32 microfracture densities for some fracture dipsets were jumping to extreme values (&gt;1E8), after the dipsets were deactivated. This was occurring because when the dipsets were deactivated, CurrentFractureData.gamma_InvBeta_M was being set to zero but Cum_Gamma_Mminus1 (and Cum_HalfLength_Mminus1) were not being reset, so were retaining anomalously high values.</t>
   </si>
 </sst>
 </file>
@@ -2502,7 +2523,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4893,6 +4914,52 @@
       </c>
       <c r="I99" s="3" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" s="6" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>623</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="F100" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H100" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A101" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C101" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="F101" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified code in GridblockConfiguration.CalculateFractureData() that calls the function FractureSet.CheckFractureDeactivation() (line 3552) to use unconditional and (&) instead of conditional and (&&). This ensures that the FractureSet.CheckFractureDeactivation() is called for every fracture set in every timestep regardless of the value of the AllSetsDeactivated flag (B95)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8D7E890-152E-4180-9238-CD26884D5679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7392D00-BBF6-4A75-8C3B-90451DAACEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="632">
   <si>
     <t>Type</t>
   </si>
@@ -2107,6 +2107,15 @@
   </si>
   <si>
     <t>In models with obliques fractures, the uFP30 and uFP32 microfracture densities for some fracture dipsets were jumping to extreme values (&gt;1E8), after the dipsets were deactivated. This was occurring because when the dipsets were deactivated, CurrentFractureData.gamma_InvBeta_M was being set to zero but Cum_Gamma_Mminus1 (and Cum_HalfLength_Mminus1) were not being reset, so were retaining anomalously high values.</t>
+  </si>
+  <si>
+    <t>B95</t>
+  </si>
+  <si>
+    <t>Not testing every fracture set for deactivation in every timestep</t>
+  </si>
+  <si>
+    <t>The code in GridblockConfiguration.CalculateFractureData() that calls the function FractureSet.CheckFractureDeactivation() to check each fracture set is deactivated used a conditional and (&amp;&amp;) rather than an unconditional and (&amp;) to link the function call with the AllSetsDeactivated flag. As a result, as soon as one fracture set was found to be active, the CheckFractureDeactivation function would not be called for any other fracture sets, thus suppressing fracture deactivation (although fracture sets can still be deactivated in the fds.calculateTotalMacrofracturePopulation function). This can be solves by replacing the conditional and with an unconditional and so the CheckFractureDeactivation function is always called, regardless of the flag value</t>
   </si>
 </sst>
 </file>
@@ -2523,7 +2532,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -4959,6 +4968,29 @@
         <v>36</v>
       </c>
       <c r="I101" s="6" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" s="6" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+      <c r="A102" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="F102" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I102" s="6" t="s">
         <v>625</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modified to take into account surface height when calculating depth at time of deformation, if the top of the Petrel grid lies above MSL (ME66)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7392D00-BBF6-4A75-8C3B-90451DAACEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D360DDB-370E-4B41-BE70-643ECFC63030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="632">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="635">
   <si>
     <t>Type</t>
   </si>
@@ -2116,6 +2116,15 @@
   </si>
   <si>
     <t>The code in GridblockConfiguration.CalculateFractureData() that calls the function FractureSet.CheckFractureDeactivation() to check each fracture set is deactivated used a conditional and (&amp;&amp;) rather than an unconditional and (&amp;) to link the function call with the AllSetsDeactivated flag. As a result, as soon as one fracture set was found to be active, the CheckFractureDeactivation function would not be called for any other fracture sets, thus suppressing fracture deactivation (although fracture sets can still be deactivated in the fds.calculateTotalMacrofracturePopulation function). This can be solves by replacing the conditional and with an unconditional and so the CheckFractureDeactivation function is always called, regardless of the flag value</t>
+  </si>
+  <si>
+    <t>ME66</t>
+  </si>
+  <si>
+    <t>Take account of surface height when calculating in situ stress</t>
+  </si>
+  <si>
+    <t>For onshore models we need to take account of the surface height when calculating lithostatic stress. Therefore if the top of the Petrel grid is above MSL we should include this height when calculating depth at time of deformation for the DFM Generator gridblock. NB If the top of the Petrel grid does not extend to the surface, the surface height above MSL will need to be included manually by calculating a depth at time of deformation property.</t>
   </si>
 </sst>
 </file>
@@ -5005,7 +5014,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6368,6 +6377,29 @@
         <v>36</v>
       </c>
       <c r="I58" s="6" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="F59" s="6">
+        <v>1</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>604</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed bugs in algorithm for calculating size and connectivity corrected fracture permeability tensor (eg B96)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D360DDB-370E-4B41-BE70-643ECFC63030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5AEDBE-76E3-4BD1-8C6F-2E8F05C4883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="638">
   <si>
     <t>Type</t>
   </si>
@@ -2125,6 +2125,15 @@
   </si>
   <si>
     <t>For onshore models we need to take account of the surface height when calculating lithostatic stress. Therefore if the top of the Petrel grid is above MSL we should include this height when calculating depth at time of deformation for the DFM Generator gridblock. NB If the top of the Petrel grid does not extend to the surface, the surface height above MSL will need to be included manually by calculating a depth at time of deformation property.</t>
+  </si>
+  <si>
+    <t>B96</t>
+  </si>
+  <si>
+    <t>Generating NaN values for porosity and permeability for uniform and size-dependent fracture aperture</t>
+  </si>
+  <si>
+    <t>The problem occurred where the stress tensor was isotropic and the present-day stress was used. The function gbc.SetFractureApertureControlData() gets a NaN from PresentDayStress.GetMinimumHorizontalAzimuth(), which then causes NaN to be returned when calculating the aperture and aperture mutlipliers based on fracture orientation. Can be fixed by using the gbc.Hmin_azimuth when GetMinimumHorizontalAzimuth(0 returns NaN - this is always defined</t>
   </si>
 </sst>
 </file>
@@ -2541,7 +2550,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -5000,6 +5009,29 @@
         <v>36</v>
       </c>
       <c r="I102" s="6" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="F103" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I103" s="6" t="s">
         <v>625</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Read Property data for dynamic loads as an alternative to simulation results, and allow effective stress to be read as well as absolute stress (ME67).
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5AEDBE-76E3-4BD1-8C6F-2E8F05C4883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E276E88-FB21-4195-9741-EA2DEE8FE167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="641">
   <si>
     <t>Type</t>
   </si>
@@ -2134,6 +2134,15 @@
   </si>
   <si>
     <t>The problem occurred where the stress tensor was isotropic and the present-day stress was used. The function gbc.SetFractureApertureControlData() gets a NaN from PresentDayStress.GetMinimumHorizontalAzimuth(), which then causes NaN to be returned when calculating the aperture and aperture mutlipliers based on fracture orientation. Can be fixed by using the gbc.Hmin_azimuth when GetMinimumHorizontalAzimuth(0 returns NaN - this is always defined</t>
+  </si>
+  <si>
+    <t>ME67</t>
+  </si>
+  <si>
+    <t>In the Petrel version, read Property data for dynamic loads as an alternative to simulation results - this allows stress tensor output from Tectonic Models (fault-related stress) to be used directly. Also, allow effective stress to be read as well as absolute stress.</t>
+  </si>
+  <si>
+    <t>Read Property data for dynamic loads as an alternative to simulation results.</t>
   </si>
 </sst>
 </file>
@@ -5046,7 +5055,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6432,6 +6441,29 @@
         <v>36</v>
       </c>
       <c r="I59" s="6" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="F60" s="6">
+        <v>3</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I60" s="6" t="s">
         <v>604</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Petrel plug-in to give user option to allow fractures to propagate across faulted gridblock boundaries (ME68)
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E276E88-FB21-4195-9741-EA2DEE8FE167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEDE256-18FD-443C-A92F-DE40C0617965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1263" uniqueCount="645">
   <si>
     <t>Type</t>
   </si>
@@ -2143,6 +2143,18 @@
   </si>
   <si>
     <t>Read Property data for dynamic loads as an alternative to simulation results.</t>
+  </si>
+  <si>
+    <t>ME68</t>
+  </si>
+  <si>
+    <t>Minor Enhancement</t>
+  </si>
+  <si>
+    <t>Allow option to ignore faults when propagating fractures</t>
+  </si>
+  <si>
+    <t>Create an option to allow fractures to propagate across faults in the Petrel version. By default fractures will terminate if they intersect a fault at a cell boundary. This can cause problems with stairstep grids contining inclined faults or faults at different depths, as any pillar intersecting a fault will cause fractures to terminate, even if the fault does not cut the layer containing the fractures. This can be presented by ensuring all neighbouring gridblocks are connected, even those where Petrel records a faulted cell boundary.</t>
   </si>
 </sst>
 </file>
@@ -5055,7 +5067,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6464,6 +6476,29 @@
         <v>36</v>
       </c>
       <c r="I60" s="6" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>643</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="F61" s="6">
+        <v>3</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I61" s="6" t="s">
         <v>604</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Petrel code to improve labelling and data recording of implicit data folders and DFNs for deformation episodes; in particular to label folders/DFNs with deformation episode number when outputting one stage per deformation episode, and adding end time to the data written to the Comments tab of the folders/DFNs (ME69). Also fixed a bug causing a crash whenever a static load deformation episode was followed by a dynamic load deformation episode (B97).
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joint\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E276E88-FB21-4195-9741-EA2DEE8FE167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0CD1F9-4150-4FE1-8C95-4FBD774A26A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="648">
   <si>
     <t>Type</t>
   </si>
@@ -2143,6 +2143,27 @@
   </si>
   <si>
     <t>Read Property data for dynamic loads as an alternative to simulation results.</t>
+  </si>
+  <si>
+    <t>ME69</t>
+  </si>
+  <si>
+    <t>Improve labelling and data recorded for intermediate implicit output and DFNs</t>
+  </si>
+  <si>
+    <t>Done in geothermal version (2.4); needs testing</t>
+  </si>
+  <si>
+    <t>In the Petrel version, when outputting an intermediate stages for each deformation episode, label the stages with the deformation episode name and number. Also record the end time for each output stage (intermediate and final) in the list of data written to the Comments tab of the top level property folder and DFN.</t>
+  </si>
+  <si>
+    <t>B97</t>
+  </si>
+  <si>
+    <t>Throwing an Index out of range exception when a static load deformation episode is followed by a dynamic load deformation episode</t>
+  </si>
+  <si>
+    <t>The Petrel version was crashing and throwing an Index out of range exception when generating the generalInputParams string describing the input parameters, if a static load deformation episode is followed by a dynamic load deformation episode. This is because it is not filling the Sij_result_list and FluidPressure_result_list with placeholder null values when creating static load deformation episode. The problem was fixed by modifying the code to do this.</t>
   </si>
 </sst>
 </file>
@@ -2559,7 +2580,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -5044,6 +5065,29 @@
         <v>625</v>
       </c>
     </row>
+    <row r="104" spans="1:9" s="6" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="F104" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>625</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <printOptions headings="1"/>
@@ -5055,7 +5099,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -6464,7 +6508,30 @@
         <v>36</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>604</v>
+        <v>643</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="F62" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I62" s="6" t="s">
+        <v>643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ongoing work on GRDECL interface (AF11). New project created. Not completed.
</commit_message>
<xml_diff>
--- a/Documentation/WorkToDo.xlsx
+++ b/Documentation/WorkToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWelch\source\repos\DFMGenerator_Code\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACEF3B6-79F6-450C-92FB-A01355673170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A12DAA-1B70-48E1-8599-30FB0F8B5FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug fixes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1281" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1288" uniqueCount="659">
   <si>
     <t>Type</t>
   </si>
@@ -2070,9 +2070,6 @@
     <t>When the driving stress is zero, and gamma^(1/beta) is zero, the fds.calculateTotalMicrofracturePopulation() was not incrementing the static microfracture population, even though microfractures could still be deactivated by growth of stress shadows around macrofractures from other dipsets. Active microfracture density was decreased, so total microfracture density was decreasing in inactive fracture dipsets. This was fixed by modifying the fds.calculateTotalMicrofracturePopulation() function to calculate s_uFP30 increment even if ts_gamma_InvBeta_N is zero.</t>
   </si>
   <si>
-    <t>Update doucmentation for v2.3</t>
-  </si>
-  <si>
     <t>Update run-through guide for v2.3 - especially section on outputting permeability tensors</t>
   </si>
   <si>
@@ -2185,6 +2182,21 @@
   </si>
   <si>
     <t>The Petrel version was assigning uniform aperture values to all fractures, regardless of orientation, even though the Barton-Bandis algorithm was selected with an anisotropic present-day stress defined (which should give an orientation-dependent fracture aperture). This was due to two bugs: 1) The ExecuteSimple() function was not correctly assigning the InitialStressRelaxation from the Stress state tab if an override was not specified in the Present Day Stress dialog, and 2) a bug in the fds.getMeanMacrofractureAperture() and similar functions used the tensile normal stress on the fracture rather than the compressive normal stress to calculate aperture.</t>
+  </si>
+  <si>
+    <t>Update documentation for v2.3</t>
+  </si>
+  <si>
+    <t>AF11</t>
+  </si>
+  <si>
+    <t>Interface with GRDECL files</t>
+  </si>
+  <si>
+    <t>Allow the standalone version of DFM Generator to read from and write to GRDECL files. Provide a user interface that allows it to fit into GRDECL-based workflows with sedimentary and diagenetic modelling packages.</t>
+  </si>
+  <si>
+    <t>Done in professional version - needs copying across</t>
   </si>
 </sst>
 </file>
@@ -4996,16 +5008,16 @@
     </row>
     <row r="100" spans="1:9" s="6" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C100" s="7" t="s">
         <v>621</v>
       </c>
-      <c r="B100" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C100" s="7" t="s">
+      <c r="D100" s="7" t="s">
         <v>622</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>623</v>
       </c>
       <c r="F100" s="6">
         <v>0.5</v>
@@ -5014,21 +5026,21 @@
         <v>36</v>
       </c>
       <c r="I100" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="101" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C101" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C101" s="7" t="s">
+      <c r="D101" s="7" t="s">
         <v>626</v>
-      </c>
-      <c r="D101" s="7" t="s">
-        <v>627</v>
       </c>
       <c r="F101" s="6">
         <v>0.5</v>
@@ -5037,21 +5049,21 @@
         <v>36</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="102" spans="1:9" s="6" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C102" s="7" t="s">
         <v>628</v>
       </c>
-      <c r="B102" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C102" s="7" t="s">
+      <c r="D102" s="7" t="s">
         <v>629</v>
-      </c>
-      <c r="D102" s="7" t="s">
-        <v>630</v>
       </c>
       <c r="F102" s="6">
         <v>0.5</v>
@@ -5060,21 +5072,21 @@
         <v>36</v>
       </c>
       <c r="I102" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="103" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C103" s="7" t="s">
         <v>634</v>
       </c>
-      <c r="B103" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C103" s="7" t="s">
+      <c r="D103" s="7" t="s">
         <v>635</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>636</v>
       </c>
       <c r="F103" s="6">
         <v>0.5</v>
@@ -5083,21 +5095,21 @@
         <v>36</v>
       </c>
       <c r="I103" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="104" spans="1:9" s="6" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C104" s="7" t="s">
         <v>644</v>
       </c>
-      <c r="B104" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C104" s="7" t="s">
+      <c r="D104" s="7" t="s">
         <v>645</v>
-      </c>
-      <c r="D104" s="7" t="s">
-        <v>646</v>
       </c>
       <c r="F104" s="6">
         <v>0.5</v>
@@ -5106,21 +5118,21 @@
         <v>36</v>
       </c>
       <c r="I104" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="105" spans="1:9" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C105" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="B105" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C105" s="7" t="s">
+      <c r="D105" s="7" t="s">
         <v>653</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>654</v>
       </c>
       <c r="F105" s="6">
         <v>1</v>
@@ -5129,7 +5141,7 @@
         <v>36</v>
       </c>
       <c r="I105" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
   </sheetData>
@@ -6414,7 +6426,7 @@
         <v>38</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -6437,7 +6449,7 @@
         <v>36</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -6460,7 +6472,7 @@
         <v>36</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6483,7 +6495,7 @@
         <v>36</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -6506,21 +6518,21 @@
         <v>36</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C59" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="D59" s="7" t="s">
         <v>632</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>633</v>
       </c>
       <c r="F59" s="6">
         <v>1</v>
@@ -6529,21 +6541,21 @@
         <v>36</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F60" s="6">
         <v>3</v>
@@ -6552,22 +6564,22 @@
         <v>36</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>640</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="C61" s="7" t="s">
         <v>641</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="D61" s="7" t="s">
         <v>642</v>
       </c>
-      <c r="D61" s="7" t="s">
-        <v>643</v>
-      </c>
       <c r="F61" s="6">
         <v>3</v>
       </c>
@@ -6575,21 +6587,21 @@
         <v>36</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C62" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>648</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>649</v>
       </c>
       <c r="F62" s="6">
         <v>0.5</v>
@@ -6598,7 +6610,7 @@
         <v>36</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
   </sheetData>
@@ -7170,24 +7182,27 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>618</v>
-      </c>
-      <c r="B23" s="8" t="s">
+    <row r="23" spans="1:9" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>617</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="13" t="s">
+        <v>654</v>
+      </c>
+      <c r="D23" s="13" t="s">
         <v>616</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>617</v>
-      </c>
-      <c r="F23" s="8">
+      <c r="F23" s="12">
         <v>1</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>36</v>
+      <c r="H23" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>658</v>
       </c>
     </row>
   </sheetData>
@@ -7199,7 +7214,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -7458,7 +7473,7 @@
         <v>37</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -7482,7 +7497,30 @@
         <v>37</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>655</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>656</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>657</v>
+      </c>
+      <c r="F12" s="12">
+        <v>10</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>619</v>
       </c>
     </row>
   </sheetData>

</xml_diff>